<commit_message>
Product Bible: source types read OOTB (iNXT BrokerVerse), BIBS (TechNXT Dev Environment), BDOI BRD/FRS
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Product_Bible/BIBS_Product_Bible_BDOI_LOB_Library_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Product_Bible/BIBS_Product_Bible_BDOI_LOB_Library_v1.0.xlsx
@@ -1299,7 +1299,7 @@
     <row r="48">
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Source legend: 'BDOI document' rows come from BDOI's BRDs / FRS; 'Market practice (to confirm with BDOI)' rows are Philippine non-life market practice and need BDOI confirmation. No BDOI-specific fact is assumed.</t>
+          <t>Source legend: 'BDOI BRD/FRS' rows come from BDOI's BRDs / FRS; 'Market practice (to confirm with BDOI)' rows are Philippine non-life market practice and need BDOI confirmation. No BDOI-specific fact is assumed.</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="S5" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="S6" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="S7" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="S11" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="S12" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="S13" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="S14" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="S15" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="S16" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="S20" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="S21" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="S23" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="S24" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="S25" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="S26" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="S28" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="S29" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="S30" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="S31" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="S33" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="S34" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -4509,7 +4509,7 @@
       </c>
       <c r="S35" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="S36" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="S37" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="S38" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="S39" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="S40" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="S41" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="S42" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="S43" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="S44" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="S45" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="S46" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="S47" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="S52" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="S53" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="S54" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
       </c>
       <c r="S55" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6546,7 +6546,7 @@
       </c>
       <c r="S56" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6643,7 +6643,7 @@
       </c>
       <c r="S57" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6740,7 +6740,7 @@
       </c>
       <c r="S58" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="S59" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7031,7 +7031,7 @@
       </c>
       <c r="S61" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="S62" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="S63" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -7322,7 +7322,7 @@
       </c>
       <c r="S64" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="S65" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="S66" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="S67" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7710,7 +7710,7 @@
       </c>
       <c r="S68" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
       </c>
       <c r="S69" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -7904,7 +7904,7 @@
       </c>
       <c r="S70" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="S71" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="S72" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="S73" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8292,7 +8292,7 @@
       </c>
       <c r="S74" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8389,7 +8389,7 @@
       </c>
       <c r="S75" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="S76" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="S77" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="S78" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -8777,7 +8777,7 @@
       </c>
       <c r="S79" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8874,7 @@
       </c>
       <c r="S80" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -8971,7 +8971,7 @@
       </c>
       <c r="S81" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -9068,7 +9068,7 @@
       </c>
       <c r="S82" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="S83" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="S84" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -9563,21 +9563,12 @@
     <mergeCell ref="A2:S2"/>
   </mergeCells>
   <conditionalFormatting sqref="S5:S587">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:S587">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13145,7 +13136,7 @@
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13168,7 @@
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13465,7 +13456,7 @@
       </c>
       <c r="F16" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13497,7 +13488,7 @@
       </c>
       <c r="F17" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13529,7 +13520,7 @@
       </c>
       <c r="F18" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13625,7 +13616,7 @@
       </c>
       <c r="F21" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -13657,7 +13648,7 @@
       </c>
       <c r="F22" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -13721,7 +13712,7 @@
       </c>
       <c r="F24" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -14467,21 +14458,12 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F547">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:F547">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14651,7 +14633,7 @@
       </c>
       <c r="J5" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -14807,7 +14789,7 @@
       </c>
       <c r="J8" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15389,21 +15371,12 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J519">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:J519">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15540,7 +15513,7 @@
       </c>
       <c r="G5" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15577,7 +15550,7 @@
       </c>
       <c r="G6" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15614,7 +15587,7 @@
       </c>
       <c r="G7" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15651,7 +15624,7 @@
       </c>
       <c r="G8" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15688,7 +15661,7 @@
       </c>
       <c r="G9" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15725,7 +15698,7 @@
       </c>
       <c r="G10" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15762,7 +15735,7 @@
       </c>
       <c r="G11" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15799,7 +15772,7 @@
       </c>
       <c r="G12" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15836,7 +15809,7 @@
       </c>
       <c r="G13" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15873,7 +15846,7 @@
       </c>
       <c r="G14" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15910,7 +15883,7 @@
       </c>
       <c r="G15" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -15947,7 +15920,7 @@
       </c>
       <c r="G16" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -15984,7 +15957,7 @@
       </c>
       <c r="G17" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16021,7 +15994,7 @@
       </c>
       <c r="G18" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16058,7 +16031,7 @@
       </c>
       <c r="G19" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16095,7 +16068,7 @@
       </c>
       <c r="G20" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16132,7 +16105,7 @@
       </c>
       <c r="G21" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16169,7 +16142,7 @@
       </c>
       <c r="G22" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16206,7 +16179,7 @@
       </c>
       <c r="G23" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16243,7 +16216,7 @@
       </c>
       <c r="G24" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16280,7 +16253,7 @@
       </c>
       <c r="G25" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16317,7 +16290,7 @@
       </c>
       <c r="G26" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16354,7 +16327,7 @@
       </c>
       <c r="G27" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16391,7 +16364,7 @@
       </c>
       <c r="G28" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16428,7 +16401,7 @@
       </c>
       <c r="G29" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16465,7 +16438,7 @@
       </c>
       <c r="G30" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16502,7 +16475,7 @@
       </c>
       <c r="G31" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16539,7 +16512,7 @@
       </c>
       <c r="G32" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16576,7 +16549,7 @@
       </c>
       <c r="G33" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -16613,7 +16586,7 @@
       </c>
       <c r="G34" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -16650,7 +16623,7 @@
       </c>
       <c r="G35" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16687,7 +16660,7 @@
       </c>
       <c r="G36" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16724,7 +16697,7 @@
       </c>
       <c r="G37" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16761,7 +16734,7 @@
       </c>
       <c r="G38" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16798,7 +16771,7 @@
       </c>
       <c r="G39" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16835,7 +16808,7 @@
       </c>
       <c r="G40" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16872,7 +16845,7 @@
       </c>
       <c r="G41" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16909,7 +16882,7 @@
       </c>
       <c r="G42" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16946,7 +16919,7 @@
       </c>
       <c r="G43" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -16983,7 +16956,7 @@
       </c>
       <c r="G44" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17020,7 +16993,7 @@
       </c>
       <c r="G45" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17057,7 +17030,7 @@
       </c>
       <c r="G46" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17094,7 +17067,7 @@
       </c>
       <c r="G47" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17131,7 +17104,7 @@
       </c>
       <c r="G48" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17168,7 +17141,7 @@
       </c>
       <c r="G49" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17205,7 +17178,7 @@
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17242,7 +17215,7 @@
       </c>
       <c r="G51" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17279,7 +17252,7 @@
       </c>
       <c r="G52" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17316,7 +17289,7 @@
       </c>
       <c r="G53" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17353,7 +17326,7 @@
       </c>
       <c r="G54" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17390,7 +17363,7 @@
       </c>
       <c r="G55" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17427,7 +17400,7 @@
       </c>
       <c r="G56" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17464,7 +17437,7 @@
       </c>
       <c r="G57" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17474,7 @@
       </c>
       <c r="G58" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17538,7 +17511,7 @@
       </c>
       <c r="G59" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17575,7 +17548,7 @@
       </c>
       <c r="G60" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17649,7 +17622,7 @@
       </c>
       <c r="G62" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17686,7 +17659,7 @@
       </c>
       <c r="G63" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -17760,7 +17733,7 @@
       </c>
       <c r="G65" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -17797,7 +17770,7 @@
       </c>
       <c r="G66" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
     </row>
@@ -17807,21 +17780,12 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="G5:G566">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:G566">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18565,21 +18529,12 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H519">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:H519">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19406,7 +19361,7 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -19423,7 +19378,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -19950,7 +19905,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -19980,7 +19935,7 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
@@ -20060,7 +20015,7 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
@@ -20070,12 +20025,12 @@
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
@@ -20085,7 +20040,7 @@
       </c>
       <c r="AH1" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="AI1" t="inlineStr">
@@ -20127,7 +20082,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -20157,7 +20112,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -20237,7 +20192,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -20247,12 +20202,12 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -20262,7 +20217,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -20304,7 +20259,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -20334,7 +20289,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -20414,7 +20369,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -20424,12 +20379,12 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
@@ -20439,12 +20394,12 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
     </row>
@@ -20531,7 +20486,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>OOTB reference</t>
+          <t>OOTB (iNXT BrokerVerse)</t>
         </is>
       </c>
     </row>
@@ -21722,7 +21677,7 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>Where the product comes from: BDOI document, BIBS configuration or market practice</t>
+          <t>Where the product comes from: BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB or market practice</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr"/>
@@ -21745,7 +21700,7 @@
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -22705,7 +22660,7 @@
       </c>
       <c r="D93" s="12" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -23165,7 +23120,7 @@
       </c>
       <c r="D115" s="12" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -23353,7 +23308,7 @@
       </c>
       <c r="D125" s="12" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -23483,7 +23438,7 @@
       </c>
       <c r="D132" s="14" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -23635,7 +23590,7 @@
       </c>
       <c r="D140" s="14" t="inlineStr">
         <is>
-          <t>BDOI document, BIBS configuration, OOTB reference, Market practice (to confirm with BDOI)</t>
+          <t>BDOI BRD/FRS, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice (to confirm with BDOI)</t>
         </is>
       </c>
     </row>
@@ -23693,7 +23648,7 @@
       </c>
       <c r="D143" s="12" t="inlineStr">
         <is>
-          <t>Source document, Programme deliverable, BIBS configuration, OOTB reference, Market practice, Assumption (market practice), Open question for BDOI</t>
+          <t>Source document, Programme deliverable, BIBS (TechNXT Dev Environment), OOTB (iNXT BrokerVerse), Market practice, Assumption (market practice), Open question for BDOI</t>
         </is>
       </c>
     </row>
@@ -23860,7 +23815,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -23897,7 +23852,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -23934,7 +23889,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -23971,7 +23926,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24008,7 +23963,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24045,7 +24000,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24082,7 +24037,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24119,7 +24074,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24156,7 +24111,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24193,7 +24148,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24230,7 +24185,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24267,7 +24222,7 @@
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24304,7 +24259,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24341,7 +24296,7 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24378,7 +24333,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24415,7 +24370,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24452,7 +24407,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24489,7 +24444,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24526,7 +24481,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24563,7 +24518,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24600,7 +24555,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24637,7 +24592,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24674,7 +24629,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24711,7 +24666,7 @@
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24748,7 +24703,7 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24785,7 +24740,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24822,7 +24777,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24859,7 +24814,7 @@
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24896,7 +24851,7 @@
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24933,7 +24888,7 @@
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -24970,7 +24925,7 @@
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25007,7 +24962,7 @@
       </c>
       <c r="G36" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25044,7 +24999,7 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25081,7 +25036,7 @@
       </c>
       <c r="G38" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25118,7 +25073,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25155,7 +25110,7 @@
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25192,7 +25147,7 @@
       </c>
       <c r="G41" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25229,7 +25184,7 @@
       </c>
       <c r="G42" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25266,7 +25221,7 @@
       </c>
       <c r="G43" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25303,7 +25258,7 @@
       </c>
       <c r="G44" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25340,7 +25295,7 @@
       </c>
       <c r="G45" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25377,7 +25332,7 @@
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25414,7 +25369,7 @@
       </c>
       <c r="G47" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25451,7 +25406,7 @@
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25488,7 +25443,7 @@
       </c>
       <c r="G49" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25525,7 +25480,7 @@
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25562,7 +25517,7 @@
       </c>
       <c r="G51" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25599,7 +25554,7 @@
       </c>
       <c r="G52" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25636,7 +25591,7 @@
       </c>
       <c r="G53" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25673,7 +25628,7 @@
       </c>
       <c r="G54" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25710,7 +25665,7 @@
       </c>
       <c r="G55" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25747,7 +25702,7 @@
       </c>
       <c r="G56" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25784,7 +25739,7 @@
       </c>
       <c r="G57" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25821,7 +25776,7 @@
       </c>
       <c r="G58" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25858,7 +25813,7 @@
       </c>
       <c r="G59" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25895,7 +25850,7 @@
       </c>
       <c r="G60" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25932,7 +25887,7 @@
       </c>
       <c r="G61" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -25969,7 +25924,7 @@
       </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26006,7 +25961,7 @@
       </c>
       <c r="G63" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26043,7 +25998,7 @@
       </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26080,7 +26035,7 @@
       </c>
       <c r="G65" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26117,7 +26072,7 @@
       </c>
       <c r="G66" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26154,7 +26109,7 @@
       </c>
       <c r="G67" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26191,7 +26146,7 @@
       </c>
       <c r="G68" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26228,7 +26183,7 @@
       </c>
       <c r="G69" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26265,7 +26220,7 @@
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26302,7 +26257,7 @@
       </c>
       <c r="G71" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26339,7 +26294,7 @@
       </c>
       <c r="G72" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26376,7 +26331,7 @@
       </c>
       <c r="G73" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26413,7 +26368,7 @@
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26450,7 +26405,7 @@
       </c>
       <c r="G75" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26487,7 +26442,7 @@
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26524,7 +26479,7 @@
       </c>
       <c r="G77" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26561,7 +26516,7 @@
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26598,7 +26553,7 @@
       </c>
       <c r="G79" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26635,7 +26590,7 @@
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26672,7 +26627,7 @@
       </c>
       <c r="G81" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26709,7 +26664,7 @@
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26746,7 +26701,7 @@
       </c>
       <c r="G83" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26783,7 +26738,7 @@
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -26820,7 +26775,7 @@
       </c>
       <c r="G85" s="12" t="inlineStr">
         <is>
-          <t>OOTB reference data (read 12-Oct-2026)</t>
+          <t>OOTB (iNXT BrokerVerse), read 12-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -27012,7 +26967,7 @@
       </c>
       <c r="K5" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27069,7 +27024,7 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27126,7 +27081,7 @@
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27183,7 +27138,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27240,7 +27195,7 @@
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27297,7 +27252,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27354,7 +27309,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27411,7 +27366,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27468,7 +27423,7 @@
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27525,7 +27480,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27582,7 +27537,7 @@
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27639,7 +27594,7 @@
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27696,7 +27651,7 @@
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27753,7 +27708,7 @@
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27810,7 +27765,7 @@
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -27867,7 +27822,7 @@
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -27924,7 +27879,7 @@
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -27981,7 +27936,7 @@
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -28038,7 +27993,7 @@
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -28095,7 +28050,7 @@
       </c>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28152,7 +28107,7 @@
       </c>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28209,7 +28164,7 @@
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28266,7 +28221,7 @@
       </c>
       <c r="K27" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28323,7 +28278,7 @@
       </c>
       <c r="K28" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28380,7 +28335,7 @@
       </c>
       <c r="K29" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -28437,7 +28392,7 @@
       </c>
       <c r="K30" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28494,7 +28449,7 @@
       </c>
       <c r="K31" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28506,7 @@
       </c>
       <c r="K32" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28608,7 +28563,7 @@
       </c>
       <c r="K33" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28665,7 +28620,7 @@
       </c>
       <c r="K34" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28722,7 +28677,7 @@
       </c>
       <c r="K35" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -28779,7 +28734,7 @@
       </c>
       <c r="K36" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28836,7 +28791,7 @@
       </c>
       <c r="K37" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28893,7 +28848,7 @@
       </c>
       <c r="K38" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -28950,7 +28905,7 @@
       </c>
       <c r="K39" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29007,7 +28962,7 @@
       </c>
       <c r="K40" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29064,7 +29019,7 @@
       </c>
       <c r="K41" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29121,7 +29076,7 @@
       </c>
       <c r="K42" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29178,7 +29133,7 @@
       </c>
       <c r="K43" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29235,7 +29190,7 @@
       </c>
       <c r="K44" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29292,7 +29247,7 @@
       </c>
       <c r="K45" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29349,7 +29304,7 @@
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29406,7 +29361,7 @@
       </c>
       <c r="K47" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29463,7 +29418,7 @@
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29520,7 +29475,7 @@
       </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29577,7 +29532,7 @@
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29634,7 +29589,7 @@
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29691,7 +29646,7 @@
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29748,7 +29703,7 @@
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29805,7 +29760,7 @@
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29862,7 +29817,7 @@
       </c>
       <c r="K55" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29919,7 +29874,7 @@
       </c>
       <c r="K56" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -29976,7 +29931,7 @@
       </c>
       <c r="K57" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30033,7 +29988,7 @@
       </c>
       <c r="K58" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30090,7 +30045,7 @@
       </c>
       <c r="K59" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30147,7 +30102,7 @@
       </c>
       <c r="K60" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30204,7 +30159,7 @@
       </c>
       <c r="K61" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30261,7 +30216,7 @@
       </c>
       <c r="K62" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30318,7 +30273,7 @@
       </c>
       <c r="K63" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30375,7 +30330,7 @@
       </c>
       <c r="K64" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30432,7 +30387,7 @@
       </c>
       <c r="K65" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -30489,7 +30444,7 @@
       </c>
       <c r="K66" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -30546,7 +30501,7 @@
       </c>
       <c r="K67" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30558,7 @@
       </c>
       <c r="K68" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -30660,7 +30615,7 @@
       </c>
       <c r="K69" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (package versions)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (package versions)</t>
         </is>
       </c>
     </row>
@@ -30717,7 +30672,7 @@
       </c>
       <c r="K70" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30774,7 +30729,7 @@
       </c>
       <c r="K71" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30831,7 +30786,7 @@
       </c>
       <c r="K72" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30888,7 +30843,7 @@
       </c>
       <c r="K73" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -30945,7 +30900,7 @@
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -31002,7 +30957,7 @@
       </c>
       <c r="K75" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -31059,7 +31014,7 @@
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -31116,7 +31071,7 @@
       </c>
       <c r="K77" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration (Employee Benefits)</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue (Employee Benefits)</t>
         </is>
       </c>
     </row>
@@ -31173,7 +31128,7 @@
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31230,7 +31185,7 @@
       </c>
       <c r="K79" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31287,7 +31242,7 @@
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31344,7 +31299,7 @@
       </c>
       <c r="K81" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31401,7 +31356,7 @@
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31458,7 +31413,7 @@
       </c>
       <c r="K83" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31515,7 +31470,7 @@
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31572,7 +31527,7 @@
       </c>
       <c r="K85" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31629,7 +31584,7 @@
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31686,7 +31641,7 @@
       </c>
       <c r="K87" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31743,7 +31698,7 @@
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31800,7 +31755,7 @@
       </c>
       <c r="K89" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31857,7 +31812,7 @@
       </c>
       <c r="K90" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31914,7 +31869,7 @@
       </c>
       <c r="K91" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -31971,7 +31926,7 @@
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32028,7 +31983,7 @@
       </c>
       <c r="K93" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32085,7 +32040,7 @@
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32142,7 +32097,7 @@
       </c>
       <c r="K95" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32199,7 +32154,7 @@
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32256,7 +32211,7 @@
       </c>
       <c r="K97" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32313,7 +32268,7 @@
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32370,7 +32325,7 @@
       </c>
       <c r="K99" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32427,7 +32382,7 @@
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32439,7 @@
       </c>
       <c r="K101" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32541,7 +32496,7 @@
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32598,7 +32553,7 @@
       </c>
       <c r="K103" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32610,7 @@
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32712,7 +32667,7 @@
       </c>
       <c r="K105" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32769,7 +32724,7 @@
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32826,7 +32781,7 @@
       </c>
       <c r="K107" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32883,7 +32838,7 @@
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32940,7 +32895,7 @@
       </c>
       <c r="K109" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -32997,7 +32952,7 @@
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33054,7 +33009,7 @@
       </c>
       <c r="K111" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33111,7 +33066,7 @@
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33168,7 +33123,7 @@
       </c>
       <c r="K113" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33225,7 +33180,7 @@
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33282,7 +33237,7 @@
       </c>
       <c r="K115" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33339,7 +33294,7 @@
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33396,7 +33351,7 @@
       </c>
       <c r="K117" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33453,7 +33408,7 @@
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33510,7 +33465,7 @@
       </c>
       <c r="K119" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33567,7 +33522,7 @@
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33624,7 +33579,7 @@
       </c>
       <c r="K121" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33681,7 +33636,7 @@
       </c>
       <c r="K122" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33738,7 +33693,7 @@
       </c>
       <c r="K123" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33795,7 +33750,7 @@
       </c>
       <c r="K124" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33852,7 +33807,7 @@
       </c>
       <c r="K125" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33909,7 +33864,7 @@
       </c>
       <c r="K126" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -33966,7 +33921,7 @@
       </c>
       <c r="K127" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34023,7 +33978,7 @@
       </c>
       <c r="K128" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34080,7 +34035,7 @@
       </c>
       <c r="K129" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34137,7 +34092,7 @@
       </c>
       <c r="K130" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34194,7 +34149,7 @@
       </c>
       <c r="K131" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34251,7 +34206,7 @@
       </c>
       <c r="K132" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34308,7 +34263,7 @@
       </c>
       <c r="K133" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34365,7 +34320,7 @@
       </c>
       <c r="K134" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34422,7 +34377,7 @@
       </c>
       <c r="K135" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34479,7 +34434,7 @@
       </c>
       <c r="K136" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34536,7 +34491,7 @@
       </c>
       <c r="K137" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34593,7 +34548,7 @@
       </c>
       <c r="K138" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34650,7 +34605,7 @@
       </c>
       <c r="K139" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34707,7 +34662,7 @@
       </c>
       <c r="K140" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34764,7 +34719,7 @@
       </c>
       <c r="K141" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34821,7 +34776,7 @@
       </c>
       <c r="K142" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34878,7 +34833,7 @@
       </c>
       <c r="K143" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34935,7 +34890,7 @@
       </c>
       <c r="K144" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -34992,7 +34947,7 @@
       </c>
       <c r="K145" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35049,7 +35004,7 @@
       </c>
       <c r="K146" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35106,7 +35061,7 @@
       </c>
       <c r="K147" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35163,7 +35118,7 @@
       </c>
       <c r="K148" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35220,7 +35175,7 @@
       </c>
       <c r="K149" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35277,7 +35232,7 @@
       </c>
       <c r="K150" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35334,7 +35289,7 @@
       </c>
       <c r="K151" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35391,7 +35346,7 @@
       </c>
       <c r="K152" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35448,7 +35403,7 @@
       </c>
       <c r="K153" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35505,7 +35460,7 @@
       </c>
       <c r="K154" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35562,7 +35517,7 @@
       </c>
       <c r="K155" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35619,7 +35574,7 @@
       </c>
       <c r="K156" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35676,7 +35631,7 @@
       </c>
       <c r="K157" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35733,7 +35688,7 @@
       </c>
       <c r="K158" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35790,7 +35745,7 @@
       </c>
       <c r="K159" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35847,7 +35802,7 @@
       </c>
       <c r="K160" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35904,7 +35859,7 @@
       </c>
       <c r="K161" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -35961,7 +35916,7 @@
       </c>
       <c r="K162" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36018,7 +35973,7 @@
       </c>
       <c r="K163" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36075,7 +36030,7 @@
       </c>
       <c r="K164" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36132,7 +36087,7 @@
       </c>
       <c r="K165" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36189,7 +36144,7 @@
       </c>
       <c r="K166" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36246,7 +36201,7 @@
       </c>
       <c r="K167" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36303,7 +36258,7 @@
       </c>
       <c r="K168" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36360,7 +36315,7 @@
       </c>
       <c r="K169" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36417,7 +36372,7 @@
       </c>
       <c r="K170" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36474,7 +36429,7 @@
       </c>
       <c r="K171" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36531,7 +36486,7 @@
       </c>
       <c r="K172" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36588,7 +36543,7 @@
       </c>
       <c r="K173" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36600,7 @@
       </c>
       <c r="K174" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36702,7 +36657,7 @@
       </c>
       <c r="K175" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36759,7 +36714,7 @@
       </c>
       <c r="K176" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36816,7 +36771,7 @@
       </c>
       <c r="K177" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36873,7 +36828,7 @@
       </c>
       <c r="K178" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36930,7 +36885,7 @@
       </c>
       <c r="K179" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -36987,7 +36942,7 @@
       </c>
       <c r="K180" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37044,7 +36999,7 @@
       </c>
       <c r="K181" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37101,7 +37056,7 @@
       </c>
       <c r="K182" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37158,7 +37113,7 @@
       </c>
       <c r="K183" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37215,7 +37170,7 @@
       </c>
       <c r="K184" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37272,7 +37227,7 @@
       </c>
       <c r="K185" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37329,7 +37284,7 @@
       </c>
       <c r="K186" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37386,7 +37341,7 @@
       </c>
       <c r="K187" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37443,7 +37398,7 @@
       </c>
       <c r="K188" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37500,7 +37455,7 @@
       </c>
       <c r="K189" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37557,7 +37512,7 @@
       </c>
       <c r="K190" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37569,7 @@
       </c>
       <c r="K191" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37671,7 +37626,7 @@
       </c>
       <c r="K192" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37728,7 +37683,7 @@
       </c>
       <c r="K193" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37785,7 +37740,7 @@
       </c>
       <c r="K194" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37842,7 +37797,7 @@
       </c>
       <c r="K195" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37899,7 +37854,7 @@
       </c>
       <c r="K196" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -37956,7 +37911,7 @@
       </c>
       <c r="K197" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38013,7 +37968,7 @@
       </c>
       <c r="K198" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38070,7 +38025,7 @@
       </c>
       <c r="K199" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38082,7 @@
       </c>
       <c r="K200" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38184,7 +38139,7 @@
       </c>
       <c r="K201" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38241,7 +38196,7 @@
       </c>
       <c r="K202" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38298,7 +38253,7 @@
       </c>
       <c r="K203" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38355,7 +38310,7 @@
       </c>
       <c r="K204" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -38412,7 +38367,7 @@
       </c>
       <c r="K205" s="12" t="inlineStr">
         <is>
-          <t>BIBS catalogue configuration</t>
+          <t>BIBS (TechNXT Dev Environment) catalogue</t>
         </is>
       </c>
     </row>
@@ -39640,7 +39595,7 @@
       </c>
       <c r="G5" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -39682,7 +39637,7 @@
       </c>
       <c r="G6" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -39724,7 +39679,7 @@
       </c>
       <c r="G7" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -39892,7 +39847,7 @@
       </c>
       <c r="G11" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
@@ -39934,7 +39889,7 @@
       </c>
       <c r="G12" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -39976,7 +39931,7 @@
       </c>
       <c r="G13" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -40018,7 +39973,7 @@
       </c>
       <c r="G14" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -40060,7 +40015,7 @@
       </c>
       <c r="G15" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -40102,7 +40057,7 @@
       </c>
       <c r="G16" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
@@ -40228,7 +40183,7 @@
       </c>
       <c r="G19" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -40270,7 +40225,7 @@
       </c>
       <c r="G20" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -40312,7 +40267,7 @@
       </c>
       <c r="G21" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -40354,7 +40309,7 @@
       </c>
       <c r="G22" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -40480,7 +40435,7 @@
       </c>
       <c r="G25" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -40522,7 +40477,7 @@
       </c>
       <c r="G26" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -40606,7 +40561,7 @@
       </c>
       <c r="G28" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H28" s="12" t="inlineStr">
@@ -40648,7 +40603,7 @@
       </c>
       <c r="G29" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
@@ -40690,7 +40645,7 @@
       </c>
       <c r="G30" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H30" s="12" t="inlineStr">
@@ -40732,7 +40687,7 @@
       </c>
       <c r="G31" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
@@ -40816,7 +40771,7 @@
       </c>
       <c r="G33" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
@@ -40900,7 +40855,7 @@
       </c>
       <c r="G35" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
@@ -40942,7 +40897,7 @@
       </c>
       <c r="G36" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H36" s="12" t="inlineStr">
@@ -40984,7 +40939,7 @@
       </c>
       <c r="G37" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
@@ -41026,7 +40981,7 @@
       </c>
       <c r="G38" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H38" s="12" t="inlineStr">
@@ -41068,7 +41023,7 @@
       </c>
       <c r="G39" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr">
@@ -41110,7 +41065,7 @@
       </c>
       <c r="G40" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H40" s="12" t="inlineStr">
@@ -41152,7 +41107,7 @@
       </c>
       <c r="G41" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H41" s="12" t="inlineStr">
@@ -41194,7 +41149,7 @@
       </c>
       <c r="G42" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H42" s="12" t="inlineStr">
@@ -41236,7 +41191,7 @@
       </c>
       <c r="G43" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
@@ -41278,7 +41233,7 @@
       </c>
       <c r="G44" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H44" s="12" t="inlineStr">
@@ -41320,7 +41275,7 @@
       </c>
       <c r="G45" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
@@ -41362,7 +41317,7 @@
       </c>
       <c r="G46" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H46" s="12" t="inlineStr">
@@ -41404,7 +41359,7 @@
       </c>
       <c r="G47" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
@@ -41446,7 +41401,7 @@
       </c>
       <c r="G48" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H48" s="12" t="inlineStr">
@@ -41488,7 +41443,7 @@
       </c>
       <c r="G49" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H49" s="12" t="inlineStr">
@@ -41530,7 +41485,7 @@
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H50" s="12" t="inlineStr">
@@ -41740,7 +41695,7 @@
       </c>
       <c r="G55" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H55" s="12" t="inlineStr">
@@ -41782,7 +41737,7 @@
       </c>
       <c r="G56" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H56" s="12" t="inlineStr">
@@ -41824,7 +41779,7 @@
       </c>
       <c r="G57" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H57" s="12" t="inlineStr">
@@ -41866,7 +41821,7 @@
       </c>
       <c r="G58" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H58" s="12" t="inlineStr">
@@ -41908,7 +41863,7 @@
       </c>
       <c r="G59" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H59" s="12" t="inlineStr">
@@ -41950,7 +41905,7 @@
       </c>
       <c r="G60" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H60" s="12" t="inlineStr">
@@ -41992,7 +41947,7 @@
       </c>
       <c r="G61" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H61" s="12" t="inlineStr">
@@ -42034,7 +41989,7 @@
       </c>
       <c r="G62" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H62" s="12" t="inlineStr">
@@ -42118,7 +42073,7 @@
       </c>
       <c r="G64" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H64" s="12" t="inlineStr">
@@ -42160,7 +42115,7 @@
       </c>
       <c r="G65" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H65" s="12" t="inlineStr">
@@ -42202,7 +42157,7 @@
       </c>
       <c r="G66" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H66" s="12" t="inlineStr">
@@ -42244,7 +42199,7 @@
       </c>
       <c r="G67" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H67" s="12" t="inlineStr">
@@ -42286,7 +42241,7 @@
       </c>
       <c r="G68" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H68" s="12" t="inlineStr">
@@ -42328,7 +42283,7 @@
       </c>
       <c r="G69" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
@@ -42370,7 +42325,7 @@
       </c>
       <c r="G70" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H70" s="12" t="inlineStr">
@@ -42412,7 +42367,7 @@
       </c>
       <c r="G71" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H71" s="12" t="inlineStr">
@@ -42454,7 +42409,7 @@
       </c>
       <c r="G72" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H72" s="12" t="inlineStr">
@@ -42496,7 +42451,7 @@
       </c>
       <c r="G73" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H73" s="12" t="inlineStr">
@@ -42538,7 +42493,7 @@
       </c>
       <c r="G74" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H74" s="12" t="inlineStr">
@@ -42580,7 +42535,7 @@
       </c>
       <c r="G75" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H75" s="12" t="inlineStr">
@@ -42622,7 +42577,7 @@
       </c>
       <c r="G76" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H76" s="12" t="inlineStr">
@@ -42664,7 +42619,7 @@
       </c>
       <c r="G77" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H77" s="12" t="inlineStr">
@@ -42706,7 +42661,7 @@
       </c>
       <c r="G78" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H78" s="12" t="inlineStr">
@@ -42748,7 +42703,7 @@
       </c>
       <c r="G79" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H79" s="12" t="inlineStr">
@@ -42790,7 +42745,7 @@
       </c>
       <c r="G80" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H80" s="12" t="inlineStr">
@@ -42832,7 +42787,7 @@
       </c>
       <c r="G81" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H81" s="12" t="inlineStr">
@@ -42874,7 +42829,7 @@
       </c>
       <c r="G82" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H82" s="12" t="inlineStr">
@@ -42916,7 +42871,7 @@
       </c>
       <c r="G83" s="28" t="inlineStr">
         <is>
-          <t>BDOI document</t>
+          <t>BDOI BRD/FRS</t>
         </is>
       </c>
       <c r="H83" s="12" t="inlineStr">
@@ -42958,7 +42913,7 @@
       </c>
       <c r="G84" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H84" s="12" t="inlineStr">
@@ -43000,7 +42955,7 @@
       </c>
       <c r="G85" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr">
@@ -43042,7 +42997,7 @@
       </c>
       <c r="G86" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H86" s="12" t="inlineStr">
@@ -43084,7 +43039,7 @@
       </c>
       <c r="G87" s="28" t="inlineStr">
         <is>
-          <t>BIBS configuration</t>
+          <t>BIBS (TechNXT Dev Environment)</t>
         </is>
       </c>
       <c r="H87" s="12" t="inlineStr">
@@ -43239,21 +43194,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G590">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1" stopIfTrue="1">
-      <formula>"BDOI document"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"BIBS configuration"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"OOTB reference"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Market practice (to confirm with BDOI)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:H590">
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" priority="6" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>